<commit_message>
Approve Ch1 Discussion 1; make it the reference teaching Short
- CLAUDE.md, make-short skill, style guide, build_edl.py: tao-ch1-passionless-subtle
  is the reference spec
- no opening title by default; full proposed transcript approved before cutting;
  titles written to grip a general YouTube audience; QA checks for keyed,
  centred images and live fades
- schedule: Ch1 Discussion 1 Ready, 'Why Trying Harder Makes You Miss What Matters'

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0124jWQy9r2ao2voUGSjfXFK
</commit_message>
<xml_diff>
--- a/docs/release-schedule.xlsx
+++ b/docs/release-schedule.xlsx
@@ -784,20 +784,22 @@
       </c>
       <c r="J3" s="18" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="K3" s="18" t="inlineStr">
         <is>
-          <t>Passionless, You See the Subtle · Tao Te Ching, Ch. 1</t>
+          <t>Why Trying Harder Makes You Miss What Matters</t>
         </is>
       </c>
       <c r="L3" s="18" t="inlineStr">
         <is>
-          <t>Main teaching: always passionless, observe the subtle; ever intent, observe the apparent; you need both (shorts/tao-ch1-passionless-subtle). Made, awaiting review.</t>
-        </is>
-      </c>
-      <c r="M3" s="23" t="n"/>
+          <t>Main teaching: always passionless, observe the subtle; ever intent, observe the apparent; you need both (shorts/tao-ch1-passionless-subtle). Made, awaiting review.; main teaching: always passionless, observe the subtle; ever intent, observe the apparent</t>
+        </is>
+      </c>
+      <c r="M3" s="23" t="n">
+        <v>46319</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="16">
       <c r="A4" s="18" t="n">

</xml_diff>

<commit_message>
Ch1 Discussion 2: 'A way can be a guide, not a fixed path'
- shorts/tao-ch1-fixed-path: spec, EDL, images, thumbnails, delivery notes
- audio.py: peak target -1.3 dBTP so the AAC file stays at or under -1
- schedule: Ch1 D1 released, D2 in progress
- shorts/tao-ch1-names-labels: spec for the bonus 'names' Short (in progress)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0124jWQy9r2ao2voUGSjfXFK
</commit_message>
<xml_diff>
--- a/docs/release-schedule.xlsx
+++ b/docs/release-schedule.xlsx
@@ -784,7 +784,7 @@
       </c>
       <c r="J3" s="18" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>Released</t>
         </is>
       </c>
       <c r="K3" s="18" t="inlineStr">
@@ -841,12 +841,20 @@
       </c>
       <c r="J4" s="18" t="inlineStr">
         <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="K4" s="18" t="n"/>
-      <c r="L4" s="18" t="n"/>
-      <c r="M4" s="20" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Turn It Into a Formula and It Loses Its Power</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>a way can be a guide, not a fixed path</t>
+        </is>
+      </c>
+      <c r="M4" s="23" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="16">
       <c r="A5" s="18" t="n">

</xml_diff>